<commit_message>
Text bugs and issues.
</commit_message>
<xml_diff>
--- a/final_documents/Courses_List.xlsx
+++ b/final_documents/Courses_List.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,10 +55,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -439,7 +442,7 @@
     <col width="3" customWidth="1" min="5" max="5"/>
     <col width="3" customWidth="1" min="6" max="6"/>
     <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,130 +456,130 @@
           <t>Course Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Course Category</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>ECE000</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Semiconductor Physics</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>PCM</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ECE001</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Fundamentals of Semiconductor Physics for VLSI Laboratory</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>PCM</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3" t="n">
+      <c r="D3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>5</v>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ECE002</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Course 2</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>PCM</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="4" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>